<commit_message>
entradas 24/09: stock ERP (captura + stock_diario) y exports de Aloha BR/PY y OTROS (sesion peer)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/stock/stock_diario.xlsx
+++ b/fuentes/stock/stock_diario.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\poronga\fuentes\stock\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\PorongaEnLaNube\gonza_pepe\fuentes\stock\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{09416FA0-9E7E-4B23-914F-0A3DADD8E451}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F547EA98-6E22-4017-9802-0E4BBC3C4A50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{4FFBE23B-D66B-4748-9C46-355EF952DEC4}"/>
   </bookViews>
   <sheets>
     <sheet name="stock" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="21">
   <si>
     <t>fecha</t>
   </si>
@@ -82,6 +82,12 @@
   </si>
   <si>
     <t>captura ERP 19/09 cierre (2026-09-19_stock_erp_captura.jpeg)</t>
+  </si>
+  <si>
+    <t>24/09/2026</t>
+  </si>
+  <si>
+    <t>captura ERP 24/09 15:45 (2026-09-24_stock_erp_captura.jpeg)</t>
   </si>
 </sst>
 </file>
@@ -91,7 +97,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -129,10 +135,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="164" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
-    <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -447,15 +453,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{457B4668-4E99-47AC-A4C5-38EAADC6154A}">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" customWidth="1" style="3"/>
+    <col min="1" max="1" width="12.7109375" style="3" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" customWidth="1"/>
     <col min="6" max="6" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -477,280 +483,371 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="0">
+      <c r="C2">
         <v>21026</v>
       </c>
-      <c r="D2" s="0">
+      <c r="D2">
         <v>22</v>
       </c>
-      <c r="E2" s="0">
+      <c r="E2">
         <f>ROUND(C2/D2,0)</f>
         <v>956</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="0">
+      <c r="C3">
         <v>23023</v>
       </c>
-      <c r="D3" s="0">
+      <c r="D3">
         <v>19</v>
       </c>
-      <c r="E3" s="0">
+      <c r="E3">
         <f>ROUND(C3/D3,0)</f>
         <v>1212</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="0">
+      <c r="C4">
         <v>10628</v>
       </c>
-      <c r="D4" s="0">
+      <c r="D4">
         <v>22</v>
       </c>
-      <c r="E4" s="0">
+      <c r="E4">
         <f>ROUND(C4/D4,0)</f>
         <v>483</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="0">
+      <c r="C5">
         <v>1958</v>
       </c>
-      <c r="D5" s="0">
+      <c r="D5">
         <v>20</v>
       </c>
-      <c r="E5" s="0">
+      <c r="E5">
         <f>ROUND(C5/D5,0)</f>
         <v>98</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="0">
+      <c r="C6">
         <v>19725</v>
       </c>
-      <c r="D6" s="0">
+      <c r="D6">
         <v>22</v>
       </c>
-      <c r="E6" s="0">
+      <c r="E6">
         <v>897</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="0" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7">
+      <c r="G6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="0">
+      <c r="C7">
         <v>22081</v>
       </c>
-      <c r="D7" s="0">
+      <c r="D7">
         <v>19</v>
       </c>
-      <c r="E7" s="0">
+      <c r="E7">
         <v>1162</v>
       </c>
-      <c r="F7" s="0" t="s">
+      <c r="F7" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="0" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8">
+      <c r="G7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="0">
+      <c r="C8">
         <v>11881</v>
       </c>
-      <c r="D8" s="0">
+      <c r="D8">
         <v>22</v>
       </c>
-      <c r="E8" s="0">
+      <c r="E8">
         <v>540</v>
       </c>
-      <c r="F8" s="0" t="s">
+      <c r="F8" t="s">
         <v>15</v>
       </c>
-      <c r="G8" s="0" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9">
+      <c r="G8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="0">
+      <c r="C9">
         <v>1844</v>
       </c>
-      <c r="D9" s="0">
+      <c r="D9">
         <v>20</v>
       </c>
-      <c r="E9" s="0">
+      <c r="E9">
         <v>92</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="F9" t="s">
         <v>15</v>
       </c>
-      <c r="G9" s="0" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10">
+      <c r="G9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="0">
+      <c r="C10">
         <v>15893</v>
       </c>
-      <c r="D10" s="0">
+      <c r="D10">
         <v>22</v>
       </c>
-      <c r="E10" s="0">
+      <c r="E10">
         <v>722</v>
       </c>
-      <c r="F10" s="0" t="s">
+      <c r="F10" t="s">
         <v>18</v>
       </c>
-      <c r="G10" s="0" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11">
+      <c r="G10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="0">
+      <c r="C11">
         <v>20033</v>
       </c>
-      <c r="D11" s="0">
+      <c r="D11">
         <v>19</v>
       </c>
-      <c r="E11" s="0">
+      <c r="E11">
         <v>1054</v>
       </c>
-      <c r="F11" s="0" t="s">
+      <c r="F11" t="s">
         <v>18</v>
       </c>
-      <c r="G11" s="0" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12">
+      <c r="G11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="0">
+      <c r="C12">
         <v>14132</v>
       </c>
-      <c r="D12" s="0">
+      <c r="D12">
         <v>22</v>
       </c>
-      <c r="E12" s="0">
+      <c r="E12">
         <v>642</v>
       </c>
-      <c r="F12" s="0" t="s">
+      <c r="F12" t="s">
         <v>18</v>
       </c>
-      <c r="G12" s="0" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13">
+      <c r="G12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="0">
+      <c r="C13">
         <v>1972</v>
       </c>
-      <c r="D13" s="0">
+      <c r="D13">
         <v>20</v>
       </c>
-      <c r="E13" s="0">
+      <c r="E13">
         <v>99</v>
       </c>
-      <c r="F13" s="0" t="s">
+      <c r="F13" t="s">
         <v>18</v>
       </c>
-      <c r="G13" s="0" t="s">
+      <c r="G13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14">
+        <v>13757</v>
+      </c>
+      <c r="D14">
+        <v>22</v>
+      </c>
+      <c r="E14">
+        <v>625</v>
+      </c>
+      <c r="F14" t="s">
+        <v>20</v>
+      </c>
+      <c r="G14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15">
+        <v>16317</v>
+      </c>
+      <c r="D15">
+        <v>19</v>
+      </c>
+      <c r="E15">
+        <v>859</v>
+      </c>
+      <c r="F15" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16">
+        <v>12585</v>
+      </c>
+      <c r="D16">
+        <v>22</v>
+      </c>
+      <c r="E16">
+        <v>572</v>
+      </c>
+      <c r="F16" t="s">
+        <v>20</v>
+      </c>
+      <c r="G16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17">
+        <v>1610</v>
+      </c>
+      <c r="D17">
+        <v>20</v>
+      </c>
+      <c r="E17">
+        <v>81</v>
+      </c>
+      <c r="F17" t="s">
+        <v>20</v>
+      </c>
+      <c r="G17" t="s">
         <v>16</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
stock ERP 25/09: captura y 4 filas en stock_diario.xlsx (sesion peer)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/stock/stock_diario.xlsx
+++ b/fuentes/stock/stock_diario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\PorongaEnLaNube\gonza_pepe\fuentes\stock\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F547EA98-6E22-4017-9802-0E4BBC3C4A50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{102F76EF-B8F3-4E08-AC86-6CB04984EA17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{4FFBE23B-D66B-4748-9C46-355EF952DEC4}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="23">
   <si>
     <t>fecha</t>
   </si>
@@ -88,6 +88,12 @@
   </si>
   <si>
     <t>captura ERP 24/09 15:45 (2026-09-24_stock_erp_captura.jpeg)</t>
+  </si>
+  <si>
+    <t>25/09/2026</t>
+  </si>
+  <si>
+    <t>captura ERP 25/09 12:25 (2026-09-25_stock_erp_captura.jpeg)</t>
   </si>
 </sst>
 </file>
@@ -453,7 +459,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{457B4668-4E99-47AC-A4C5-38EAADC6154A}">
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="3" customWidth="1"/>
@@ -847,6 +853,98 @@
         <v>16</v>
       </c>
     </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18">
+        <v>13353</v>
+      </c>
+      <c r="D18">
+        <v>22</v>
+      </c>
+      <c r="E18">
+        <v>607</v>
+      </c>
+      <c r="F18" t="s">
+        <v>22</v>
+      </c>
+      <c r="G18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19">
+        <v>16330</v>
+      </c>
+      <c r="D19">
+        <v>19</v>
+      </c>
+      <c r="E19">
+        <v>859</v>
+      </c>
+      <c r="F19" t="s">
+        <v>22</v>
+      </c>
+      <c r="G19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20">
+        <v>15019</v>
+      </c>
+      <c r="D20">
+        <v>22</v>
+      </c>
+      <c r="E20">
+        <v>683</v>
+      </c>
+      <c r="F20" t="s">
+        <v>22</v>
+      </c>
+      <c r="G20" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C21">
+        <v>2151</v>
+      </c>
+      <c r="D21">
+        <v>20</v>
+      </c>
+      <c r="E21">
+        <v>108</v>
+      </c>
+      <c r="F21" t="s">
+        <v>22</v>
+      </c>
+      <c r="G21" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
stock ERP 26/09: captura, 4 filas en stock_diario.xlsx y 4 en ventas_erp
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes/stock/stock_diario.xlsx
+++ b/fuentes/stock/stock_diario.xlsx
@@ -15,7 +15,7 @@
   <sheets>
     <sheet name="stock" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>fecha</t>
   </si>
@@ -94,6 +94,12 @@
   </si>
   <si>
     <t>captura ERP 25/09 12:25 (2026-09-25_stock_erp_captura.jpeg)</t>
+  </si>
+  <si>
+    <t>26/09/2026</t>
+  </si>
+  <si>
+    <t>captura ERP 26/09 10:16 (2026-09-26_stock_erp_captura.jpeg)</t>
   </si>
 </sst>
 </file>
@@ -103,7 +109,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -140,11 +146,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="5">
+    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="0" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="164" applyNumberFormat="1" fontId="1" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+    <xf numFmtId="164" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -459,15 +466,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{457B4668-4E99-47AC-A4C5-38EAADC6154A}">
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" style="3" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1" style="3"/>
     <col min="2" max="2" width="10.7109375" customWidth="1"/>
     <col min="6" max="6" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -489,463 +496,556 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="0" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="0">
         <v>21026</v>
       </c>
-      <c r="D2">
-        <v>22</v>
-      </c>
-      <c r="E2">
+      <c r="D2" s="0">
+        <v>22</v>
+      </c>
+      <c r="E2" s="0">
         <f>ROUND(C2/D2,0)</f>
         <v>956</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="0" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="0">
         <v>23023</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="0">
         <v>19</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="0">
         <f>ROUND(C3/D3,0)</f>
         <v>1212</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="0" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4">
       <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="0">
         <v>10628</v>
       </c>
-      <c r="D4">
-        <v>22</v>
-      </c>
-      <c r="E4">
+      <c r="D4" s="0">
+        <v>22</v>
+      </c>
+      <c r="E4" s="0">
         <f>ROUND(C4/D4,0)</f>
         <v>483</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="0" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="0">
         <v>1958</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="0">
         <v>20</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="0">
         <f>ROUND(C5/D5,0)</f>
         <v>98</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="0" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="0">
         <v>19725</v>
       </c>
-      <c r="D6">
-        <v>22</v>
-      </c>
-      <c r="E6">
+      <c r="D6" s="0">
+        <v>22</v>
+      </c>
+      <c r="E6" s="0">
         <v>897</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="G6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G6" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="0">
         <v>22081</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="0">
         <v>19</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="0">
         <v>1162</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="G7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G7" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="0">
         <v>11881</v>
       </c>
-      <c r="D8">
-        <v>22</v>
-      </c>
-      <c r="E8">
+      <c r="D8" s="0">
+        <v>22</v>
+      </c>
+      <c r="E8" s="0">
         <v>540</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="G8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G8" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="0">
         <v>1844</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="0">
         <v>20</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="0">
         <v>92</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="G9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G9" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="0">
         <v>15893</v>
       </c>
-      <c r="D10">
-        <v>22</v>
-      </c>
-      <c r="E10">
+      <c r="D10" s="0">
+        <v>22</v>
+      </c>
+      <c r="E10" s="0">
         <v>722</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="G10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G10" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="0">
         <v>20033</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="0">
         <v>19</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="0">
         <v>1054</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="G11" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G11" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="0">
         <v>14132</v>
       </c>
-      <c r="D12">
-        <v>22</v>
-      </c>
-      <c r="E12">
+      <c r="D12" s="0">
+        <v>22</v>
+      </c>
+      <c r="E12" s="0">
         <v>642</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="G12" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G12" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="0">
         <v>1972</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="0">
         <v>20</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="0">
         <v>99</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="G13" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G13" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14">
       <c r="A14" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="0">
         <v>13757</v>
       </c>
-      <c r="D14">
-        <v>22</v>
-      </c>
-      <c r="E14">
+      <c r="D14" s="0">
+        <v>22</v>
+      </c>
+      <c r="E14" s="0">
         <v>625</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="G14" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G14" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15">
       <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="0">
         <v>16317</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="0">
         <v>19</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="0">
         <v>859</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="G15" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G15" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16">
       <c r="A16" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="0">
         <v>12585</v>
       </c>
-      <c r="D16">
-        <v>22</v>
-      </c>
-      <c r="E16">
+      <c r="D16" s="0">
+        <v>22</v>
+      </c>
+      <c r="E16" s="0">
         <v>572</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="G16" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G16" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17">
       <c r="A17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="0">
         <v>1610</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="0">
         <v>20</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="0">
         <v>81</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="G17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G17" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18">
       <c r="A18" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="0">
         <v>13353</v>
       </c>
-      <c r="D18">
-        <v>22</v>
-      </c>
-      <c r="E18">
+      <c r="D18" s="0">
+        <v>22</v>
+      </c>
+      <c r="E18" s="0">
         <v>607</v>
       </c>
-      <c r="F18" t="s">
-        <v>22</v>
-      </c>
-      <c r="G18" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F18" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="G18" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19">
       <c r="A19" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="0">
         <v>16330</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="0">
         <v>19</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="0">
         <v>859</v>
       </c>
-      <c r="F19" t="s">
-        <v>22</v>
-      </c>
-      <c r="G19" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F19" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="G19" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20">
       <c r="A20" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="0">
         <v>15019</v>
       </c>
-      <c r="D20">
-        <v>22</v>
-      </c>
-      <c r="E20">
+      <c r="D20" s="0">
+        <v>22</v>
+      </c>
+      <c r="E20" s="0">
         <v>683</v>
       </c>
-      <c r="F20" t="s">
-        <v>22</v>
-      </c>
-      <c r="G20" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F20" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="G20" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21">
       <c r="A21" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="0">
         <v>2151</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="0">
         <v>20</v>
       </c>
-      <c r="E21">
+      <c r="E21" s="0">
         <v>108</v>
       </c>
-      <c r="F21" t="s">
-        <v>22</v>
-      </c>
-      <c r="G21" t="s">
+      <c r="F21" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="G21" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="0">
+        <v>12452</v>
+      </c>
+      <c r="D22" s="0">
+        <v>22</v>
+      </c>
+      <c r="E22" s="0">
+        <v>566</v>
+      </c>
+      <c r="F22" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="G22" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="C23" s="0">
+        <v>21955</v>
+      </c>
+      <c r="D23" s="0">
+        <v>19</v>
+      </c>
+      <c r="E23" s="0">
+        <v>1156</v>
+      </c>
+      <c r="F23" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="G23" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="0">
+        <v>14786</v>
+      </c>
+      <c r="D24" s="0">
+        <v>22</v>
+      </c>
+      <c r="E24" s="0">
+        <v>672</v>
+      </c>
+      <c r="F24" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="G24" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B25" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C25" s="0">
+        <v>2017</v>
+      </c>
+      <c r="D25" s="0">
+        <v>20</v>
+      </c>
+      <c r="E25" s="0">
+        <v>101</v>
+      </c>
+      <c r="F25" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="G25" s="0" t="s">
         <v>16</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>